<commit_message>
update data formatting matching table examples
</commit_message>
<xml_diff>
--- a/data/example/data_formatting/obs_columns_matching_examples/assay_matching_table.xlsx
+++ b/data/example/data_formatting/obs_columns_matching_examples/assay_matching_table.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,46 +493,121 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>10x_5p_v1</t>
+          <t>10x_5p_v2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10x 5' v1</t>
+          <t>10x 5' v2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10x_3p_v1</t>
+          <t>10x_5p</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10x 3' v1</t>
+          <t>10x 5' transcription profiling</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10x_5p_v2</t>
+          <t>10x_5p_v1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10x 5' v2</t>
+          <t>10x 5' v1</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>10x_3p_v2/v3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10x 3' v2</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>10x_v2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10x 3' v2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>10x_3p</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10x 3' transcription profiling</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>10x_3p_v1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10x 3' v1</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>10x</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10x 3' transcription profiling</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>